<commit_message>
Menus : mise à jour du fichier de l'année (16 journées modifiées)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pzz1ScLz4UrmnfdMpaT4KK
</commit_message>
<xml_diff>
--- a/menus/menu-2025-ehpad-fam.xlsx
+++ b/menus/menu-2025-ehpad-fam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cuisine.fam\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6664E701-E1FD-4D68-B0F8-6D802A9C3295}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD6EBA14-84EF-449F-964B-37FD63C7B62D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13020" firstSheet="30" activeTab="37" xr2:uid="{154A0DB5-4115-4A51-8B51-9981251D1FF3}"/>
   </bookViews>
@@ -95,7 +95,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4523" uniqueCount="727">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4522" uniqueCount="728">
   <si>
     <t>Menu du :</t>
   </si>
@@ -2194,9 +2194,6 @@
     <t>haricots verts</t>
   </si>
   <si>
-    <t>salade italinne</t>
-  </si>
-  <si>
     <t>salade penne poulet</t>
   </si>
   <si>
@@ -2276,6 +2273,12 @@
   </si>
   <si>
     <t>Salade pois chiche</t>
+  </si>
+  <si>
+    <t xml:space="preserve">roti de porc </t>
+  </si>
+  <si>
+    <t>epinard</t>
   </si>
 </sst>
 </file>
@@ -2286,7 +2289,7 @@
     <numFmt numFmtId="164" formatCode="[$-40C]d\-mmm;@"/>
     <numFmt numFmtId="165" formatCode="[$-40C]d\-mmm\-yy;@"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2417,6 +2420,13 @@
     <font>
       <b/>
       <sz val="14"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -2782,7 +2792,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3105,6 +3115,9 @@
     </xf>
     <xf numFmtId="20" fontId="19" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -15989,7 +16002,7 @@
       <c r="C24" s="92" t="s">
         <v>6</v>
       </c>
-      <c r="D24" s="113" t="s">
+      <c r="D24" s="114" t="s">
         <v>576</v>
       </c>
       <c r="E24" s="94" t="s">
@@ -16005,7 +16018,7 @@
         <v>150</v>
       </c>
       <c r="C25" s="92"/>
-      <c r="D25" s="113"/>
+      <c r="D25" s="114"/>
       <c r="E25" s="94"/>
     </row>
     <row r="26" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -25420,7 +25433,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="109" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="C4" s="92" t="s">
         <v>6</v>
@@ -25867,321 +25880,321 @@
     <col min="3" max="3" width="13.42578125" style="42" customWidth="1"/>
     <col min="4" max="4" width="46.28515625" style="42" customWidth="1"/>
     <col min="5" max="5" width="18.28515625" style="42" customWidth="1"/>
-    <col min="257" max="257" width="12.7109375" customWidth="1"/>
-    <col min="258" max="258" width="45.7109375" customWidth="1"/>
-    <col min="259" max="259" width="14.140625" customWidth="1"/>
-    <col min="260" max="260" width="45.7109375" customWidth="1"/>
-    <col min="261" max="261" width="19.5703125" customWidth="1"/>
-    <col min="513" max="513" width="12.7109375" customWidth="1"/>
-    <col min="514" max="514" width="45.7109375" customWidth="1"/>
-    <col min="515" max="515" width="14.140625" customWidth="1"/>
-    <col min="516" max="516" width="45.7109375" customWidth="1"/>
-    <col min="517" max="517" width="19.5703125" customWidth="1"/>
-    <col min="769" max="769" width="12.7109375" customWidth="1"/>
-    <col min="770" max="770" width="45.7109375" customWidth="1"/>
-    <col min="771" max="771" width="14.140625" customWidth="1"/>
-    <col min="772" max="772" width="45.7109375" customWidth="1"/>
-    <col min="773" max="773" width="19.5703125" customWidth="1"/>
-    <col min="1025" max="1025" width="12.7109375" customWidth="1"/>
-    <col min="1026" max="1026" width="45.7109375" customWidth="1"/>
-    <col min="1027" max="1027" width="14.140625" customWidth="1"/>
-    <col min="1028" max="1028" width="45.7109375" customWidth="1"/>
-    <col min="1029" max="1029" width="19.5703125" customWidth="1"/>
-    <col min="1281" max="1281" width="12.7109375" customWidth="1"/>
-    <col min="1282" max="1282" width="45.7109375" customWidth="1"/>
-    <col min="1283" max="1283" width="14.140625" customWidth="1"/>
-    <col min="1284" max="1284" width="45.7109375" customWidth="1"/>
-    <col min="1285" max="1285" width="19.5703125" customWidth="1"/>
-    <col min="1537" max="1537" width="12.7109375" customWidth="1"/>
-    <col min="1538" max="1538" width="45.7109375" customWidth="1"/>
-    <col min="1539" max="1539" width="14.140625" customWidth="1"/>
-    <col min="1540" max="1540" width="45.7109375" customWidth="1"/>
-    <col min="1541" max="1541" width="19.5703125" customWidth="1"/>
-    <col min="1793" max="1793" width="12.7109375" customWidth="1"/>
-    <col min="1794" max="1794" width="45.7109375" customWidth="1"/>
-    <col min="1795" max="1795" width="14.140625" customWidth="1"/>
-    <col min="1796" max="1796" width="45.7109375" customWidth="1"/>
-    <col min="1797" max="1797" width="19.5703125" customWidth="1"/>
-    <col min="2049" max="2049" width="12.7109375" customWidth="1"/>
-    <col min="2050" max="2050" width="45.7109375" customWidth="1"/>
-    <col min="2051" max="2051" width="14.140625" customWidth="1"/>
-    <col min="2052" max="2052" width="45.7109375" customWidth="1"/>
-    <col min="2053" max="2053" width="19.5703125" customWidth="1"/>
-    <col min="2305" max="2305" width="12.7109375" customWidth="1"/>
-    <col min="2306" max="2306" width="45.7109375" customWidth="1"/>
-    <col min="2307" max="2307" width="14.140625" customWidth="1"/>
-    <col min="2308" max="2308" width="45.7109375" customWidth="1"/>
-    <col min="2309" max="2309" width="19.5703125" customWidth="1"/>
-    <col min="2561" max="2561" width="12.7109375" customWidth="1"/>
-    <col min="2562" max="2562" width="45.7109375" customWidth="1"/>
-    <col min="2563" max="2563" width="14.140625" customWidth="1"/>
-    <col min="2564" max="2564" width="45.7109375" customWidth="1"/>
-    <col min="2565" max="2565" width="19.5703125" customWidth="1"/>
-    <col min="2817" max="2817" width="12.7109375" customWidth="1"/>
-    <col min="2818" max="2818" width="45.7109375" customWidth="1"/>
-    <col min="2819" max="2819" width="14.140625" customWidth="1"/>
-    <col min="2820" max="2820" width="45.7109375" customWidth="1"/>
-    <col min="2821" max="2821" width="19.5703125" customWidth="1"/>
-    <col min="3073" max="3073" width="12.7109375" customWidth="1"/>
-    <col min="3074" max="3074" width="45.7109375" customWidth="1"/>
-    <col min="3075" max="3075" width="14.140625" customWidth="1"/>
-    <col min="3076" max="3076" width="45.7109375" customWidth="1"/>
-    <col min="3077" max="3077" width="19.5703125" customWidth="1"/>
-    <col min="3329" max="3329" width="12.7109375" customWidth="1"/>
-    <col min="3330" max="3330" width="45.7109375" customWidth="1"/>
-    <col min="3331" max="3331" width="14.140625" customWidth="1"/>
-    <col min="3332" max="3332" width="45.7109375" customWidth="1"/>
-    <col min="3333" max="3333" width="19.5703125" customWidth="1"/>
-    <col min="3585" max="3585" width="12.7109375" customWidth="1"/>
-    <col min="3586" max="3586" width="45.7109375" customWidth="1"/>
-    <col min="3587" max="3587" width="14.140625" customWidth="1"/>
-    <col min="3588" max="3588" width="45.7109375" customWidth="1"/>
-    <col min="3589" max="3589" width="19.5703125" customWidth="1"/>
-    <col min="3841" max="3841" width="12.7109375" customWidth="1"/>
-    <col min="3842" max="3842" width="45.7109375" customWidth="1"/>
-    <col min="3843" max="3843" width="14.140625" customWidth="1"/>
-    <col min="3844" max="3844" width="45.7109375" customWidth="1"/>
-    <col min="3845" max="3845" width="19.5703125" customWidth="1"/>
-    <col min="4097" max="4097" width="12.7109375" customWidth="1"/>
-    <col min="4098" max="4098" width="45.7109375" customWidth="1"/>
-    <col min="4099" max="4099" width="14.140625" customWidth="1"/>
-    <col min="4100" max="4100" width="45.7109375" customWidth="1"/>
-    <col min="4101" max="4101" width="19.5703125" customWidth="1"/>
-    <col min="4353" max="4353" width="12.7109375" customWidth="1"/>
-    <col min="4354" max="4354" width="45.7109375" customWidth="1"/>
-    <col min="4355" max="4355" width="14.140625" customWidth="1"/>
-    <col min="4356" max="4356" width="45.7109375" customWidth="1"/>
-    <col min="4357" max="4357" width="19.5703125" customWidth="1"/>
-    <col min="4609" max="4609" width="12.7109375" customWidth="1"/>
-    <col min="4610" max="4610" width="45.7109375" customWidth="1"/>
-    <col min="4611" max="4611" width="14.140625" customWidth="1"/>
-    <col min="4612" max="4612" width="45.7109375" customWidth="1"/>
-    <col min="4613" max="4613" width="19.5703125" customWidth="1"/>
-    <col min="4865" max="4865" width="12.7109375" customWidth="1"/>
-    <col min="4866" max="4866" width="45.7109375" customWidth="1"/>
-    <col min="4867" max="4867" width="14.140625" customWidth="1"/>
-    <col min="4868" max="4868" width="45.7109375" customWidth="1"/>
-    <col min="4869" max="4869" width="19.5703125" customWidth="1"/>
-    <col min="5121" max="5121" width="12.7109375" customWidth="1"/>
-    <col min="5122" max="5122" width="45.7109375" customWidth="1"/>
-    <col min="5123" max="5123" width="14.140625" customWidth="1"/>
-    <col min="5124" max="5124" width="45.7109375" customWidth="1"/>
-    <col min="5125" max="5125" width="19.5703125" customWidth="1"/>
-    <col min="5377" max="5377" width="12.7109375" customWidth="1"/>
-    <col min="5378" max="5378" width="45.7109375" customWidth="1"/>
-    <col min="5379" max="5379" width="14.140625" customWidth="1"/>
-    <col min="5380" max="5380" width="45.7109375" customWidth="1"/>
-    <col min="5381" max="5381" width="19.5703125" customWidth="1"/>
-    <col min="5633" max="5633" width="12.7109375" customWidth="1"/>
-    <col min="5634" max="5634" width="45.7109375" customWidth="1"/>
-    <col min="5635" max="5635" width="14.140625" customWidth="1"/>
-    <col min="5636" max="5636" width="45.7109375" customWidth="1"/>
-    <col min="5637" max="5637" width="19.5703125" customWidth="1"/>
-    <col min="5889" max="5889" width="12.7109375" customWidth="1"/>
-    <col min="5890" max="5890" width="45.7109375" customWidth="1"/>
-    <col min="5891" max="5891" width="14.140625" customWidth="1"/>
-    <col min="5892" max="5892" width="45.7109375" customWidth="1"/>
-    <col min="5893" max="5893" width="19.5703125" customWidth="1"/>
-    <col min="6145" max="6145" width="12.7109375" customWidth="1"/>
-    <col min="6146" max="6146" width="45.7109375" customWidth="1"/>
-    <col min="6147" max="6147" width="14.140625" customWidth="1"/>
-    <col min="6148" max="6148" width="45.7109375" customWidth="1"/>
-    <col min="6149" max="6149" width="19.5703125" customWidth="1"/>
-    <col min="6401" max="6401" width="12.7109375" customWidth="1"/>
-    <col min="6402" max="6402" width="45.7109375" customWidth="1"/>
-    <col min="6403" max="6403" width="14.140625" customWidth="1"/>
-    <col min="6404" max="6404" width="45.7109375" customWidth="1"/>
-    <col min="6405" max="6405" width="19.5703125" customWidth="1"/>
-    <col min="6657" max="6657" width="12.7109375" customWidth="1"/>
-    <col min="6658" max="6658" width="45.7109375" customWidth="1"/>
-    <col min="6659" max="6659" width="14.140625" customWidth="1"/>
-    <col min="6660" max="6660" width="45.7109375" customWidth="1"/>
-    <col min="6661" max="6661" width="19.5703125" customWidth="1"/>
-    <col min="6913" max="6913" width="12.7109375" customWidth="1"/>
-    <col min="6914" max="6914" width="45.7109375" customWidth="1"/>
-    <col min="6915" max="6915" width="14.140625" customWidth="1"/>
-    <col min="6916" max="6916" width="45.7109375" customWidth="1"/>
-    <col min="6917" max="6917" width="19.5703125" customWidth="1"/>
-    <col min="7169" max="7169" width="12.7109375" customWidth="1"/>
-    <col min="7170" max="7170" width="45.7109375" customWidth="1"/>
-    <col min="7171" max="7171" width="14.140625" customWidth="1"/>
-    <col min="7172" max="7172" width="45.7109375" customWidth="1"/>
-    <col min="7173" max="7173" width="19.5703125" customWidth="1"/>
-    <col min="7425" max="7425" width="12.7109375" customWidth="1"/>
-    <col min="7426" max="7426" width="45.7109375" customWidth="1"/>
-    <col min="7427" max="7427" width="14.140625" customWidth="1"/>
-    <col min="7428" max="7428" width="45.7109375" customWidth="1"/>
-    <col min="7429" max="7429" width="19.5703125" customWidth="1"/>
-    <col min="7681" max="7681" width="12.7109375" customWidth="1"/>
-    <col min="7682" max="7682" width="45.7109375" customWidth="1"/>
-    <col min="7683" max="7683" width="14.140625" customWidth="1"/>
-    <col min="7684" max="7684" width="45.7109375" customWidth="1"/>
-    <col min="7685" max="7685" width="19.5703125" customWidth="1"/>
-    <col min="7937" max="7937" width="12.7109375" customWidth="1"/>
-    <col min="7938" max="7938" width="45.7109375" customWidth="1"/>
-    <col min="7939" max="7939" width="14.140625" customWidth="1"/>
-    <col min="7940" max="7940" width="45.7109375" customWidth="1"/>
-    <col min="7941" max="7941" width="19.5703125" customWidth="1"/>
-    <col min="8193" max="8193" width="12.7109375" customWidth="1"/>
-    <col min="8194" max="8194" width="45.7109375" customWidth="1"/>
-    <col min="8195" max="8195" width="14.140625" customWidth="1"/>
-    <col min="8196" max="8196" width="45.7109375" customWidth="1"/>
-    <col min="8197" max="8197" width="19.5703125" customWidth="1"/>
-    <col min="8449" max="8449" width="12.7109375" customWidth="1"/>
-    <col min="8450" max="8450" width="45.7109375" customWidth="1"/>
-    <col min="8451" max="8451" width="14.140625" customWidth="1"/>
-    <col min="8452" max="8452" width="45.7109375" customWidth="1"/>
-    <col min="8453" max="8453" width="19.5703125" customWidth="1"/>
-    <col min="8705" max="8705" width="12.7109375" customWidth="1"/>
-    <col min="8706" max="8706" width="45.7109375" customWidth="1"/>
-    <col min="8707" max="8707" width="14.140625" customWidth="1"/>
-    <col min="8708" max="8708" width="45.7109375" customWidth="1"/>
-    <col min="8709" max="8709" width="19.5703125" customWidth="1"/>
-    <col min="8961" max="8961" width="12.7109375" customWidth="1"/>
-    <col min="8962" max="8962" width="45.7109375" customWidth="1"/>
-    <col min="8963" max="8963" width="14.140625" customWidth="1"/>
-    <col min="8964" max="8964" width="45.7109375" customWidth="1"/>
-    <col min="8965" max="8965" width="19.5703125" customWidth="1"/>
-    <col min="9217" max="9217" width="12.7109375" customWidth="1"/>
-    <col min="9218" max="9218" width="45.7109375" customWidth="1"/>
-    <col min="9219" max="9219" width="14.140625" customWidth="1"/>
-    <col min="9220" max="9220" width="45.7109375" customWidth="1"/>
-    <col min="9221" max="9221" width="19.5703125" customWidth="1"/>
-    <col min="9473" max="9473" width="12.7109375" customWidth="1"/>
-    <col min="9474" max="9474" width="45.7109375" customWidth="1"/>
-    <col min="9475" max="9475" width="14.140625" customWidth="1"/>
-    <col min="9476" max="9476" width="45.7109375" customWidth="1"/>
-    <col min="9477" max="9477" width="19.5703125" customWidth="1"/>
-    <col min="9729" max="9729" width="12.7109375" customWidth="1"/>
-    <col min="9730" max="9730" width="45.7109375" customWidth="1"/>
-    <col min="9731" max="9731" width="14.140625" customWidth="1"/>
-    <col min="9732" max="9732" width="45.7109375" customWidth="1"/>
-    <col min="9733" max="9733" width="19.5703125" customWidth="1"/>
-    <col min="9985" max="9985" width="12.7109375" customWidth="1"/>
-    <col min="9986" max="9986" width="45.7109375" customWidth="1"/>
-    <col min="9987" max="9987" width="14.140625" customWidth="1"/>
-    <col min="9988" max="9988" width="45.7109375" customWidth="1"/>
-    <col min="9989" max="9989" width="19.5703125" customWidth="1"/>
-    <col min="10241" max="10241" width="12.7109375" customWidth="1"/>
-    <col min="10242" max="10242" width="45.7109375" customWidth="1"/>
-    <col min="10243" max="10243" width="14.140625" customWidth="1"/>
-    <col min="10244" max="10244" width="45.7109375" customWidth="1"/>
-    <col min="10245" max="10245" width="19.5703125" customWidth="1"/>
-    <col min="10497" max="10497" width="12.7109375" customWidth="1"/>
-    <col min="10498" max="10498" width="45.7109375" customWidth="1"/>
-    <col min="10499" max="10499" width="14.140625" customWidth="1"/>
-    <col min="10500" max="10500" width="45.7109375" customWidth="1"/>
-    <col min="10501" max="10501" width="19.5703125" customWidth="1"/>
-    <col min="10753" max="10753" width="12.7109375" customWidth="1"/>
-    <col min="10754" max="10754" width="45.7109375" customWidth="1"/>
-    <col min="10755" max="10755" width="14.140625" customWidth="1"/>
-    <col min="10756" max="10756" width="45.7109375" customWidth="1"/>
-    <col min="10757" max="10757" width="19.5703125" customWidth="1"/>
-    <col min="11009" max="11009" width="12.7109375" customWidth="1"/>
-    <col min="11010" max="11010" width="45.7109375" customWidth="1"/>
-    <col min="11011" max="11011" width="14.140625" customWidth="1"/>
-    <col min="11012" max="11012" width="45.7109375" customWidth="1"/>
-    <col min="11013" max="11013" width="19.5703125" customWidth="1"/>
-    <col min="11265" max="11265" width="12.7109375" customWidth="1"/>
-    <col min="11266" max="11266" width="45.7109375" customWidth="1"/>
-    <col min="11267" max="11267" width="14.140625" customWidth="1"/>
-    <col min="11268" max="11268" width="45.7109375" customWidth="1"/>
-    <col min="11269" max="11269" width="19.5703125" customWidth="1"/>
-    <col min="11521" max="11521" width="12.7109375" customWidth="1"/>
-    <col min="11522" max="11522" width="45.7109375" customWidth="1"/>
-    <col min="11523" max="11523" width="14.140625" customWidth="1"/>
-    <col min="11524" max="11524" width="45.7109375" customWidth="1"/>
-    <col min="11525" max="11525" width="19.5703125" customWidth="1"/>
-    <col min="11777" max="11777" width="12.7109375" customWidth="1"/>
-    <col min="11778" max="11778" width="45.7109375" customWidth="1"/>
-    <col min="11779" max="11779" width="14.140625" customWidth="1"/>
-    <col min="11780" max="11780" width="45.7109375" customWidth="1"/>
-    <col min="11781" max="11781" width="19.5703125" customWidth="1"/>
-    <col min="12033" max="12033" width="12.7109375" customWidth="1"/>
-    <col min="12034" max="12034" width="45.7109375" customWidth="1"/>
-    <col min="12035" max="12035" width="14.140625" customWidth="1"/>
-    <col min="12036" max="12036" width="45.7109375" customWidth="1"/>
-    <col min="12037" max="12037" width="19.5703125" customWidth="1"/>
-    <col min="12289" max="12289" width="12.7109375" customWidth="1"/>
-    <col min="12290" max="12290" width="45.7109375" customWidth="1"/>
-    <col min="12291" max="12291" width="14.140625" customWidth="1"/>
-    <col min="12292" max="12292" width="45.7109375" customWidth="1"/>
-    <col min="12293" max="12293" width="19.5703125" customWidth="1"/>
-    <col min="12545" max="12545" width="12.7109375" customWidth="1"/>
-    <col min="12546" max="12546" width="45.7109375" customWidth="1"/>
-    <col min="12547" max="12547" width="14.140625" customWidth="1"/>
-    <col min="12548" max="12548" width="45.7109375" customWidth="1"/>
-    <col min="12549" max="12549" width="19.5703125" customWidth="1"/>
-    <col min="12801" max="12801" width="12.7109375" customWidth="1"/>
-    <col min="12802" max="12802" width="45.7109375" customWidth="1"/>
-    <col min="12803" max="12803" width="14.140625" customWidth="1"/>
-    <col min="12804" max="12804" width="45.7109375" customWidth="1"/>
-    <col min="12805" max="12805" width="19.5703125" customWidth="1"/>
-    <col min="13057" max="13057" width="12.7109375" customWidth="1"/>
-    <col min="13058" max="13058" width="45.7109375" customWidth="1"/>
-    <col min="13059" max="13059" width="14.140625" customWidth="1"/>
-    <col min="13060" max="13060" width="45.7109375" customWidth="1"/>
-    <col min="13061" max="13061" width="19.5703125" customWidth="1"/>
-    <col min="13313" max="13313" width="12.7109375" customWidth="1"/>
-    <col min="13314" max="13314" width="45.7109375" customWidth="1"/>
-    <col min="13315" max="13315" width="14.140625" customWidth="1"/>
-    <col min="13316" max="13316" width="45.7109375" customWidth="1"/>
-    <col min="13317" max="13317" width="19.5703125" customWidth="1"/>
-    <col min="13569" max="13569" width="12.7109375" customWidth="1"/>
-    <col min="13570" max="13570" width="45.7109375" customWidth="1"/>
-    <col min="13571" max="13571" width="14.140625" customWidth="1"/>
-    <col min="13572" max="13572" width="45.7109375" customWidth="1"/>
-    <col min="13573" max="13573" width="19.5703125" customWidth="1"/>
-    <col min="13825" max="13825" width="12.7109375" customWidth="1"/>
-    <col min="13826" max="13826" width="45.7109375" customWidth="1"/>
-    <col min="13827" max="13827" width="14.140625" customWidth="1"/>
-    <col min="13828" max="13828" width="45.7109375" customWidth="1"/>
-    <col min="13829" max="13829" width="19.5703125" customWidth="1"/>
-    <col min="14081" max="14081" width="12.7109375" customWidth="1"/>
-    <col min="14082" max="14082" width="45.7109375" customWidth="1"/>
-    <col min="14083" max="14083" width="14.140625" customWidth="1"/>
-    <col min="14084" max="14084" width="45.7109375" customWidth="1"/>
-    <col min="14085" max="14085" width="19.5703125" customWidth="1"/>
-    <col min="14337" max="14337" width="12.7109375" customWidth="1"/>
-    <col min="14338" max="14338" width="45.7109375" customWidth="1"/>
-    <col min="14339" max="14339" width="14.140625" customWidth="1"/>
-    <col min="14340" max="14340" width="45.7109375" customWidth="1"/>
-    <col min="14341" max="14341" width="19.5703125" customWidth="1"/>
-    <col min="14593" max="14593" width="12.7109375" customWidth="1"/>
-    <col min="14594" max="14594" width="45.7109375" customWidth="1"/>
-    <col min="14595" max="14595" width="14.140625" customWidth="1"/>
-    <col min="14596" max="14596" width="45.7109375" customWidth="1"/>
-    <col min="14597" max="14597" width="19.5703125" customWidth="1"/>
-    <col min="14849" max="14849" width="12.7109375" customWidth="1"/>
-    <col min="14850" max="14850" width="45.7109375" customWidth="1"/>
-    <col min="14851" max="14851" width="14.140625" customWidth="1"/>
-    <col min="14852" max="14852" width="45.7109375" customWidth="1"/>
-    <col min="14853" max="14853" width="19.5703125" customWidth="1"/>
-    <col min="15105" max="15105" width="12.7109375" customWidth="1"/>
-    <col min="15106" max="15106" width="45.7109375" customWidth="1"/>
-    <col min="15107" max="15107" width="14.140625" customWidth="1"/>
-    <col min="15108" max="15108" width="45.7109375" customWidth="1"/>
-    <col min="15109" max="15109" width="19.5703125" customWidth="1"/>
-    <col min="15361" max="15361" width="12.7109375" customWidth="1"/>
-    <col min="15362" max="15362" width="45.7109375" customWidth="1"/>
-    <col min="15363" max="15363" width="14.140625" customWidth="1"/>
-    <col min="15364" max="15364" width="45.7109375" customWidth="1"/>
-    <col min="15365" max="15365" width="19.5703125" customWidth="1"/>
-    <col min="15617" max="15617" width="12.7109375" customWidth="1"/>
-    <col min="15618" max="15618" width="45.7109375" customWidth="1"/>
-    <col min="15619" max="15619" width="14.140625" customWidth="1"/>
-    <col min="15620" max="15620" width="45.7109375" customWidth="1"/>
-    <col min="15621" max="15621" width="19.5703125" customWidth="1"/>
-    <col min="15873" max="15873" width="12.7109375" customWidth="1"/>
-    <col min="15874" max="15874" width="45.7109375" customWidth="1"/>
-    <col min="15875" max="15875" width="14.140625" customWidth="1"/>
-    <col min="15876" max="15876" width="45.7109375" customWidth="1"/>
-    <col min="15877" max="15877" width="19.5703125" customWidth="1"/>
-    <col min="16129" max="16129" width="12.7109375" customWidth="1"/>
-    <col min="16130" max="16130" width="45.7109375" customWidth="1"/>
-    <col min="16131" max="16131" width="14.140625" customWidth="1"/>
-    <col min="16132" max="16132" width="45.7109375" customWidth="1"/>
-    <col min="16133" max="16133" width="19.5703125" customWidth="1"/>
+    <col min="256" max="256" width="12.7109375" customWidth="1"/>
+    <col min="257" max="257" width="45.7109375" customWidth="1"/>
+    <col min="258" max="258" width="14.140625" customWidth="1"/>
+    <col min="259" max="259" width="45.7109375" customWidth="1"/>
+    <col min="260" max="260" width="19.5703125" customWidth="1"/>
+    <col min="512" max="512" width="12.7109375" customWidth="1"/>
+    <col min="513" max="513" width="45.7109375" customWidth="1"/>
+    <col min="514" max="514" width="14.140625" customWidth="1"/>
+    <col min="515" max="515" width="45.7109375" customWidth="1"/>
+    <col min="516" max="516" width="19.5703125" customWidth="1"/>
+    <col min="768" max="768" width="12.7109375" customWidth="1"/>
+    <col min="769" max="769" width="45.7109375" customWidth="1"/>
+    <col min="770" max="770" width="14.140625" customWidth="1"/>
+    <col min="771" max="771" width="45.7109375" customWidth="1"/>
+    <col min="772" max="772" width="19.5703125" customWidth="1"/>
+    <col min="1024" max="1024" width="12.7109375" customWidth="1"/>
+    <col min="1025" max="1025" width="45.7109375" customWidth="1"/>
+    <col min="1026" max="1026" width="14.140625" customWidth="1"/>
+    <col min="1027" max="1027" width="45.7109375" customWidth="1"/>
+    <col min="1028" max="1028" width="19.5703125" customWidth="1"/>
+    <col min="1280" max="1280" width="12.7109375" customWidth="1"/>
+    <col min="1281" max="1281" width="45.7109375" customWidth="1"/>
+    <col min="1282" max="1282" width="14.140625" customWidth="1"/>
+    <col min="1283" max="1283" width="45.7109375" customWidth="1"/>
+    <col min="1284" max="1284" width="19.5703125" customWidth="1"/>
+    <col min="1536" max="1536" width="12.7109375" customWidth="1"/>
+    <col min="1537" max="1537" width="45.7109375" customWidth="1"/>
+    <col min="1538" max="1538" width="14.140625" customWidth="1"/>
+    <col min="1539" max="1539" width="45.7109375" customWidth="1"/>
+    <col min="1540" max="1540" width="19.5703125" customWidth="1"/>
+    <col min="1792" max="1792" width="12.7109375" customWidth="1"/>
+    <col min="1793" max="1793" width="45.7109375" customWidth="1"/>
+    <col min="1794" max="1794" width="14.140625" customWidth="1"/>
+    <col min="1795" max="1795" width="45.7109375" customWidth="1"/>
+    <col min="1796" max="1796" width="19.5703125" customWidth="1"/>
+    <col min="2048" max="2048" width="12.7109375" customWidth="1"/>
+    <col min="2049" max="2049" width="45.7109375" customWidth="1"/>
+    <col min="2050" max="2050" width="14.140625" customWidth="1"/>
+    <col min="2051" max="2051" width="45.7109375" customWidth="1"/>
+    <col min="2052" max="2052" width="19.5703125" customWidth="1"/>
+    <col min="2304" max="2304" width="12.7109375" customWidth="1"/>
+    <col min="2305" max="2305" width="45.7109375" customWidth="1"/>
+    <col min="2306" max="2306" width="14.140625" customWidth="1"/>
+    <col min="2307" max="2307" width="45.7109375" customWidth="1"/>
+    <col min="2308" max="2308" width="19.5703125" customWidth="1"/>
+    <col min="2560" max="2560" width="12.7109375" customWidth="1"/>
+    <col min="2561" max="2561" width="45.7109375" customWidth="1"/>
+    <col min="2562" max="2562" width="14.140625" customWidth="1"/>
+    <col min="2563" max="2563" width="45.7109375" customWidth="1"/>
+    <col min="2564" max="2564" width="19.5703125" customWidth="1"/>
+    <col min="2816" max="2816" width="12.7109375" customWidth="1"/>
+    <col min="2817" max="2817" width="45.7109375" customWidth="1"/>
+    <col min="2818" max="2818" width="14.140625" customWidth="1"/>
+    <col min="2819" max="2819" width="45.7109375" customWidth="1"/>
+    <col min="2820" max="2820" width="19.5703125" customWidth="1"/>
+    <col min="3072" max="3072" width="12.7109375" customWidth="1"/>
+    <col min="3073" max="3073" width="45.7109375" customWidth="1"/>
+    <col min="3074" max="3074" width="14.140625" customWidth="1"/>
+    <col min="3075" max="3075" width="45.7109375" customWidth="1"/>
+    <col min="3076" max="3076" width="19.5703125" customWidth="1"/>
+    <col min="3328" max="3328" width="12.7109375" customWidth="1"/>
+    <col min="3329" max="3329" width="45.7109375" customWidth="1"/>
+    <col min="3330" max="3330" width="14.140625" customWidth="1"/>
+    <col min="3331" max="3331" width="45.7109375" customWidth="1"/>
+    <col min="3332" max="3332" width="19.5703125" customWidth="1"/>
+    <col min="3584" max="3584" width="12.7109375" customWidth="1"/>
+    <col min="3585" max="3585" width="45.7109375" customWidth="1"/>
+    <col min="3586" max="3586" width="14.140625" customWidth="1"/>
+    <col min="3587" max="3587" width="45.7109375" customWidth="1"/>
+    <col min="3588" max="3588" width="19.5703125" customWidth="1"/>
+    <col min="3840" max="3840" width="12.7109375" customWidth="1"/>
+    <col min="3841" max="3841" width="45.7109375" customWidth="1"/>
+    <col min="3842" max="3842" width="14.140625" customWidth="1"/>
+    <col min="3843" max="3843" width="45.7109375" customWidth="1"/>
+    <col min="3844" max="3844" width="19.5703125" customWidth="1"/>
+    <col min="4096" max="4096" width="12.7109375" customWidth="1"/>
+    <col min="4097" max="4097" width="45.7109375" customWidth="1"/>
+    <col min="4098" max="4098" width="14.140625" customWidth="1"/>
+    <col min="4099" max="4099" width="45.7109375" customWidth="1"/>
+    <col min="4100" max="4100" width="19.5703125" customWidth="1"/>
+    <col min="4352" max="4352" width="12.7109375" customWidth="1"/>
+    <col min="4353" max="4353" width="45.7109375" customWidth="1"/>
+    <col min="4354" max="4354" width="14.140625" customWidth="1"/>
+    <col min="4355" max="4355" width="45.7109375" customWidth="1"/>
+    <col min="4356" max="4356" width="19.5703125" customWidth="1"/>
+    <col min="4608" max="4608" width="12.7109375" customWidth="1"/>
+    <col min="4609" max="4609" width="45.7109375" customWidth="1"/>
+    <col min="4610" max="4610" width="14.140625" customWidth="1"/>
+    <col min="4611" max="4611" width="45.7109375" customWidth="1"/>
+    <col min="4612" max="4612" width="19.5703125" customWidth="1"/>
+    <col min="4864" max="4864" width="12.7109375" customWidth="1"/>
+    <col min="4865" max="4865" width="45.7109375" customWidth="1"/>
+    <col min="4866" max="4866" width="14.140625" customWidth="1"/>
+    <col min="4867" max="4867" width="45.7109375" customWidth="1"/>
+    <col min="4868" max="4868" width="19.5703125" customWidth="1"/>
+    <col min="5120" max="5120" width="12.7109375" customWidth="1"/>
+    <col min="5121" max="5121" width="45.7109375" customWidth="1"/>
+    <col min="5122" max="5122" width="14.140625" customWidth="1"/>
+    <col min="5123" max="5123" width="45.7109375" customWidth="1"/>
+    <col min="5124" max="5124" width="19.5703125" customWidth="1"/>
+    <col min="5376" max="5376" width="12.7109375" customWidth="1"/>
+    <col min="5377" max="5377" width="45.7109375" customWidth="1"/>
+    <col min="5378" max="5378" width="14.140625" customWidth="1"/>
+    <col min="5379" max="5379" width="45.7109375" customWidth="1"/>
+    <col min="5380" max="5380" width="19.5703125" customWidth="1"/>
+    <col min="5632" max="5632" width="12.7109375" customWidth="1"/>
+    <col min="5633" max="5633" width="45.7109375" customWidth="1"/>
+    <col min="5634" max="5634" width="14.140625" customWidth="1"/>
+    <col min="5635" max="5635" width="45.7109375" customWidth="1"/>
+    <col min="5636" max="5636" width="19.5703125" customWidth="1"/>
+    <col min="5888" max="5888" width="12.7109375" customWidth="1"/>
+    <col min="5889" max="5889" width="45.7109375" customWidth="1"/>
+    <col min="5890" max="5890" width="14.140625" customWidth="1"/>
+    <col min="5891" max="5891" width="45.7109375" customWidth="1"/>
+    <col min="5892" max="5892" width="19.5703125" customWidth="1"/>
+    <col min="6144" max="6144" width="12.7109375" customWidth="1"/>
+    <col min="6145" max="6145" width="45.7109375" customWidth="1"/>
+    <col min="6146" max="6146" width="14.140625" customWidth="1"/>
+    <col min="6147" max="6147" width="45.7109375" customWidth="1"/>
+    <col min="6148" max="6148" width="19.5703125" customWidth="1"/>
+    <col min="6400" max="6400" width="12.7109375" customWidth="1"/>
+    <col min="6401" max="6401" width="45.7109375" customWidth="1"/>
+    <col min="6402" max="6402" width="14.140625" customWidth="1"/>
+    <col min="6403" max="6403" width="45.7109375" customWidth="1"/>
+    <col min="6404" max="6404" width="19.5703125" customWidth="1"/>
+    <col min="6656" max="6656" width="12.7109375" customWidth="1"/>
+    <col min="6657" max="6657" width="45.7109375" customWidth="1"/>
+    <col min="6658" max="6658" width="14.140625" customWidth="1"/>
+    <col min="6659" max="6659" width="45.7109375" customWidth="1"/>
+    <col min="6660" max="6660" width="19.5703125" customWidth="1"/>
+    <col min="6912" max="6912" width="12.7109375" customWidth="1"/>
+    <col min="6913" max="6913" width="45.7109375" customWidth="1"/>
+    <col min="6914" max="6914" width="14.140625" customWidth="1"/>
+    <col min="6915" max="6915" width="45.7109375" customWidth="1"/>
+    <col min="6916" max="6916" width="19.5703125" customWidth="1"/>
+    <col min="7168" max="7168" width="12.7109375" customWidth="1"/>
+    <col min="7169" max="7169" width="45.7109375" customWidth="1"/>
+    <col min="7170" max="7170" width="14.140625" customWidth="1"/>
+    <col min="7171" max="7171" width="45.7109375" customWidth="1"/>
+    <col min="7172" max="7172" width="19.5703125" customWidth="1"/>
+    <col min="7424" max="7424" width="12.7109375" customWidth="1"/>
+    <col min="7425" max="7425" width="45.7109375" customWidth="1"/>
+    <col min="7426" max="7426" width="14.140625" customWidth="1"/>
+    <col min="7427" max="7427" width="45.7109375" customWidth="1"/>
+    <col min="7428" max="7428" width="19.5703125" customWidth="1"/>
+    <col min="7680" max="7680" width="12.7109375" customWidth="1"/>
+    <col min="7681" max="7681" width="45.7109375" customWidth="1"/>
+    <col min="7682" max="7682" width="14.140625" customWidth="1"/>
+    <col min="7683" max="7683" width="45.7109375" customWidth="1"/>
+    <col min="7684" max="7684" width="19.5703125" customWidth="1"/>
+    <col min="7936" max="7936" width="12.7109375" customWidth="1"/>
+    <col min="7937" max="7937" width="45.7109375" customWidth="1"/>
+    <col min="7938" max="7938" width="14.140625" customWidth="1"/>
+    <col min="7939" max="7939" width="45.7109375" customWidth="1"/>
+    <col min="7940" max="7940" width="19.5703125" customWidth="1"/>
+    <col min="8192" max="8192" width="12.7109375" customWidth="1"/>
+    <col min="8193" max="8193" width="45.7109375" customWidth="1"/>
+    <col min="8194" max="8194" width="14.140625" customWidth="1"/>
+    <col min="8195" max="8195" width="45.7109375" customWidth="1"/>
+    <col min="8196" max="8196" width="19.5703125" customWidth="1"/>
+    <col min="8448" max="8448" width="12.7109375" customWidth="1"/>
+    <col min="8449" max="8449" width="45.7109375" customWidth="1"/>
+    <col min="8450" max="8450" width="14.140625" customWidth="1"/>
+    <col min="8451" max="8451" width="45.7109375" customWidth="1"/>
+    <col min="8452" max="8452" width="19.5703125" customWidth="1"/>
+    <col min="8704" max="8704" width="12.7109375" customWidth="1"/>
+    <col min="8705" max="8705" width="45.7109375" customWidth="1"/>
+    <col min="8706" max="8706" width="14.140625" customWidth="1"/>
+    <col min="8707" max="8707" width="45.7109375" customWidth="1"/>
+    <col min="8708" max="8708" width="19.5703125" customWidth="1"/>
+    <col min="8960" max="8960" width="12.7109375" customWidth="1"/>
+    <col min="8961" max="8961" width="45.7109375" customWidth="1"/>
+    <col min="8962" max="8962" width="14.140625" customWidth="1"/>
+    <col min="8963" max="8963" width="45.7109375" customWidth="1"/>
+    <col min="8964" max="8964" width="19.5703125" customWidth="1"/>
+    <col min="9216" max="9216" width="12.7109375" customWidth="1"/>
+    <col min="9217" max="9217" width="45.7109375" customWidth="1"/>
+    <col min="9218" max="9218" width="14.140625" customWidth="1"/>
+    <col min="9219" max="9219" width="45.7109375" customWidth="1"/>
+    <col min="9220" max="9220" width="19.5703125" customWidth="1"/>
+    <col min="9472" max="9472" width="12.7109375" customWidth="1"/>
+    <col min="9473" max="9473" width="45.7109375" customWidth="1"/>
+    <col min="9474" max="9474" width="14.140625" customWidth="1"/>
+    <col min="9475" max="9475" width="45.7109375" customWidth="1"/>
+    <col min="9476" max="9476" width="19.5703125" customWidth="1"/>
+    <col min="9728" max="9728" width="12.7109375" customWidth="1"/>
+    <col min="9729" max="9729" width="45.7109375" customWidth="1"/>
+    <col min="9730" max="9730" width="14.140625" customWidth="1"/>
+    <col min="9731" max="9731" width="45.7109375" customWidth="1"/>
+    <col min="9732" max="9732" width="19.5703125" customWidth="1"/>
+    <col min="9984" max="9984" width="12.7109375" customWidth="1"/>
+    <col min="9985" max="9985" width="45.7109375" customWidth="1"/>
+    <col min="9986" max="9986" width="14.140625" customWidth="1"/>
+    <col min="9987" max="9987" width="45.7109375" customWidth="1"/>
+    <col min="9988" max="9988" width="19.5703125" customWidth="1"/>
+    <col min="10240" max="10240" width="12.7109375" customWidth="1"/>
+    <col min="10241" max="10241" width="45.7109375" customWidth="1"/>
+    <col min="10242" max="10242" width="14.140625" customWidth="1"/>
+    <col min="10243" max="10243" width="45.7109375" customWidth="1"/>
+    <col min="10244" max="10244" width="19.5703125" customWidth="1"/>
+    <col min="10496" max="10496" width="12.7109375" customWidth="1"/>
+    <col min="10497" max="10497" width="45.7109375" customWidth="1"/>
+    <col min="10498" max="10498" width="14.140625" customWidth="1"/>
+    <col min="10499" max="10499" width="45.7109375" customWidth="1"/>
+    <col min="10500" max="10500" width="19.5703125" customWidth="1"/>
+    <col min="10752" max="10752" width="12.7109375" customWidth="1"/>
+    <col min="10753" max="10753" width="45.7109375" customWidth="1"/>
+    <col min="10754" max="10754" width="14.140625" customWidth="1"/>
+    <col min="10755" max="10755" width="45.7109375" customWidth="1"/>
+    <col min="10756" max="10756" width="19.5703125" customWidth="1"/>
+    <col min="11008" max="11008" width="12.7109375" customWidth="1"/>
+    <col min="11009" max="11009" width="45.7109375" customWidth="1"/>
+    <col min="11010" max="11010" width="14.140625" customWidth="1"/>
+    <col min="11011" max="11011" width="45.7109375" customWidth="1"/>
+    <col min="11012" max="11012" width="19.5703125" customWidth="1"/>
+    <col min="11264" max="11264" width="12.7109375" customWidth="1"/>
+    <col min="11265" max="11265" width="45.7109375" customWidth="1"/>
+    <col min="11266" max="11266" width="14.140625" customWidth="1"/>
+    <col min="11267" max="11267" width="45.7109375" customWidth="1"/>
+    <col min="11268" max="11268" width="19.5703125" customWidth="1"/>
+    <col min="11520" max="11520" width="12.7109375" customWidth="1"/>
+    <col min="11521" max="11521" width="45.7109375" customWidth="1"/>
+    <col min="11522" max="11522" width="14.140625" customWidth="1"/>
+    <col min="11523" max="11523" width="45.7109375" customWidth="1"/>
+    <col min="11524" max="11524" width="19.5703125" customWidth="1"/>
+    <col min="11776" max="11776" width="12.7109375" customWidth="1"/>
+    <col min="11777" max="11777" width="45.7109375" customWidth="1"/>
+    <col min="11778" max="11778" width="14.140625" customWidth="1"/>
+    <col min="11779" max="11779" width="45.7109375" customWidth="1"/>
+    <col min="11780" max="11780" width="19.5703125" customWidth="1"/>
+    <col min="12032" max="12032" width="12.7109375" customWidth="1"/>
+    <col min="12033" max="12033" width="45.7109375" customWidth="1"/>
+    <col min="12034" max="12034" width="14.140625" customWidth="1"/>
+    <col min="12035" max="12035" width="45.7109375" customWidth="1"/>
+    <col min="12036" max="12036" width="19.5703125" customWidth="1"/>
+    <col min="12288" max="12288" width="12.7109375" customWidth="1"/>
+    <col min="12289" max="12289" width="45.7109375" customWidth="1"/>
+    <col min="12290" max="12290" width="14.140625" customWidth="1"/>
+    <col min="12291" max="12291" width="45.7109375" customWidth="1"/>
+    <col min="12292" max="12292" width="19.5703125" customWidth="1"/>
+    <col min="12544" max="12544" width="12.7109375" customWidth="1"/>
+    <col min="12545" max="12545" width="45.7109375" customWidth="1"/>
+    <col min="12546" max="12546" width="14.140625" customWidth="1"/>
+    <col min="12547" max="12547" width="45.7109375" customWidth="1"/>
+    <col min="12548" max="12548" width="19.5703125" customWidth="1"/>
+    <col min="12800" max="12800" width="12.7109375" customWidth="1"/>
+    <col min="12801" max="12801" width="45.7109375" customWidth="1"/>
+    <col min="12802" max="12802" width="14.140625" customWidth="1"/>
+    <col min="12803" max="12803" width="45.7109375" customWidth="1"/>
+    <col min="12804" max="12804" width="19.5703125" customWidth="1"/>
+    <col min="13056" max="13056" width="12.7109375" customWidth="1"/>
+    <col min="13057" max="13057" width="45.7109375" customWidth="1"/>
+    <col min="13058" max="13058" width="14.140625" customWidth="1"/>
+    <col min="13059" max="13059" width="45.7109375" customWidth="1"/>
+    <col min="13060" max="13060" width="19.5703125" customWidth="1"/>
+    <col min="13312" max="13312" width="12.7109375" customWidth="1"/>
+    <col min="13313" max="13313" width="45.7109375" customWidth="1"/>
+    <col min="13314" max="13314" width="14.140625" customWidth="1"/>
+    <col min="13315" max="13315" width="45.7109375" customWidth="1"/>
+    <col min="13316" max="13316" width="19.5703125" customWidth="1"/>
+    <col min="13568" max="13568" width="12.7109375" customWidth="1"/>
+    <col min="13569" max="13569" width="45.7109375" customWidth="1"/>
+    <col min="13570" max="13570" width="14.140625" customWidth="1"/>
+    <col min="13571" max="13571" width="45.7109375" customWidth="1"/>
+    <col min="13572" max="13572" width="19.5703125" customWidth="1"/>
+    <col min="13824" max="13824" width="12.7109375" customWidth="1"/>
+    <col min="13825" max="13825" width="45.7109375" customWidth="1"/>
+    <col min="13826" max="13826" width="14.140625" customWidth="1"/>
+    <col min="13827" max="13827" width="45.7109375" customWidth="1"/>
+    <col min="13828" max="13828" width="19.5703125" customWidth="1"/>
+    <col min="14080" max="14080" width="12.7109375" customWidth="1"/>
+    <col min="14081" max="14081" width="45.7109375" customWidth="1"/>
+    <col min="14082" max="14082" width="14.140625" customWidth="1"/>
+    <col min="14083" max="14083" width="45.7109375" customWidth="1"/>
+    <col min="14084" max="14084" width="19.5703125" customWidth="1"/>
+    <col min="14336" max="14336" width="12.7109375" customWidth="1"/>
+    <col min="14337" max="14337" width="45.7109375" customWidth="1"/>
+    <col min="14338" max="14338" width="14.140625" customWidth="1"/>
+    <col min="14339" max="14339" width="45.7109375" customWidth="1"/>
+    <col min="14340" max="14340" width="19.5703125" customWidth="1"/>
+    <col min="14592" max="14592" width="12.7109375" customWidth="1"/>
+    <col min="14593" max="14593" width="45.7109375" customWidth="1"/>
+    <col min="14594" max="14594" width="14.140625" customWidth="1"/>
+    <col min="14595" max="14595" width="45.7109375" customWidth="1"/>
+    <col min="14596" max="14596" width="19.5703125" customWidth="1"/>
+    <col min="14848" max="14848" width="12.7109375" customWidth="1"/>
+    <col min="14849" max="14849" width="45.7109375" customWidth="1"/>
+    <col min="14850" max="14850" width="14.140625" customWidth="1"/>
+    <col min="14851" max="14851" width="45.7109375" customWidth="1"/>
+    <col min="14852" max="14852" width="19.5703125" customWidth="1"/>
+    <col min="15104" max="15104" width="12.7109375" customWidth="1"/>
+    <col min="15105" max="15105" width="45.7109375" customWidth="1"/>
+    <col min="15106" max="15106" width="14.140625" customWidth="1"/>
+    <col min="15107" max="15107" width="45.7109375" customWidth="1"/>
+    <col min="15108" max="15108" width="19.5703125" customWidth="1"/>
+    <col min="15360" max="15360" width="12.7109375" customWidth="1"/>
+    <col min="15361" max="15361" width="45.7109375" customWidth="1"/>
+    <col min="15362" max="15362" width="14.140625" customWidth="1"/>
+    <col min="15363" max="15363" width="45.7109375" customWidth="1"/>
+    <col min="15364" max="15364" width="19.5703125" customWidth="1"/>
+    <col min="15616" max="15616" width="12.7109375" customWidth="1"/>
+    <col min="15617" max="15617" width="45.7109375" customWidth="1"/>
+    <col min="15618" max="15618" width="14.140625" customWidth="1"/>
+    <col min="15619" max="15619" width="45.7109375" customWidth="1"/>
+    <col min="15620" max="15620" width="19.5703125" customWidth="1"/>
+    <col min="15872" max="15872" width="12.7109375" customWidth="1"/>
+    <col min="15873" max="15873" width="45.7109375" customWidth="1"/>
+    <col min="15874" max="15874" width="14.140625" customWidth="1"/>
+    <col min="15875" max="15875" width="45.7109375" customWidth="1"/>
+    <col min="15876" max="15876" width="19.5703125" customWidth="1"/>
+    <col min="16128" max="16128" width="12.7109375" customWidth="1"/>
+    <col min="16129" max="16129" width="45.7109375" customWidth="1"/>
+    <col min="16130" max="16130" width="14.140625" customWidth="1"/>
+    <col min="16131" max="16131" width="45.7109375" customWidth="1"/>
+    <col min="16132" max="16132" width="19.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -26402,11 +26415,11 @@
     <row r="18" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="50"/>
       <c r="B18" s="97" t="s">
-        <v>626</v>
+        <v>387</v>
       </c>
       <c r="C18" s="88"/>
-      <c r="D18" s="89" t="s">
-        <v>627</v>
+      <c r="D18" s="113" t="s">
+        <v>348</v>
       </c>
       <c r="E18" s="94"/>
     </row>
@@ -26420,8 +26433,8 @@
       <c r="C19" s="92" t="s">
         <v>6</v>
       </c>
-      <c r="D19" s="93" t="s">
-        <v>44</v>
+      <c r="D19" s="108" t="s">
+        <v>694</v>
       </c>
       <c r="E19" s="94" t="s">
         <v>6</v>
@@ -26435,7 +26448,7 @@
       <c r="B20" s="95"/>
       <c r="C20" s="92"/>
       <c r="D20" s="93" t="s">
-        <v>33</v>
+        <v>569</v>
       </c>
       <c r="E20" s="94"/>
     </row>
@@ -26463,8 +26476,8 @@
     </row>
     <row r="23" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="50"/>
-      <c r="B23" s="111" t="s">
-        <v>699</v>
+      <c r="B23" s="89" t="s">
+        <v>627</v>
       </c>
       <c r="C23" s="88"/>
       <c r="D23" s="89" t="s">
@@ -26483,7 +26496,7 @@
         <v>6</v>
       </c>
       <c r="D24" s="93" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E24" s="94" t="s">
         <v>6</v>
@@ -26526,7 +26539,7 @@
     <row r="28" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="50"/>
       <c r="B28" s="97" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="C28" s="88"/>
       <c r="D28" s="89" t="s">
@@ -26544,8 +26557,8 @@
       <c r="C29" s="92" t="s">
         <v>6</v>
       </c>
-      <c r="D29" s="108" t="s">
-        <v>694</v>
+      <c r="D29" s="93" t="s">
+        <v>44</v>
       </c>
       <c r="E29" s="94" t="s">
         <v>6</v>
@@ -26561,7 +26574,7 @@
       </c>
       <c r="C30" s="92"/>
       <c r="D30" s="93" t="s">
-        <v>569</v>
+        <v>33</v>
       </c>
       <c r="E30" s="94"/>
     </row>
@@ -26657,8 +26670,8 @@
       <c r="E38" s="45"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="85" orientation="landscape" r:id="rId1"/>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -27036,7 +27049,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="109" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C4" s="92" t="s">
         <v>6</v>
@@ -27097,8 +27110,8 @@
       <c r="A9" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="93" t="s">
-        <v>703</v>
+      <c r="B9" s="95" t="s">
+        <v>648</v>
       </c>
       <c r="C9" s="92" t="s">
         <v>6</v>
@@ -27116,10 +27129,10 @@
         <v>46259</v>
       </c>
       <c r="B10" s="93" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="C10" s="92"/>
-      <c r="D10" s="93"/>
+      <c r="D10" s="95"/>
       <c r="E10" s="94"/>
     </row>
     <row r="11" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -27147,11 +27160,11 @@
     <row r="13" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="50"/>
       <c r="B13" s="97" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="C13" s="88"/>
       <c r="D13" s="110" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="E13" s="90"/>
     </row>
@@ -27160,7 +27173,7 @@
         <v>10</v>
       </c>
       <c r="B14" s="95" t="s">
-        <v>648</v>
+        <v>452</v>
       </c>
       <c r="C14" s="92" t="s">
         <v>6</v>
@@ -27177,9 +27190,6 @@
         <f>A10+1</f>
         <v>46260</v>
       </c>
-      <c r="B15" s="109" t="s">
-        <v>709</v>
-      </c>
       <c r="C15" s="92"/>
       <c r="D15" s="93"/>
       <c r="E15" s="94"/>
@@ -27213,7 +27223,7 @@
       </c>
       <c r="C18" s="88"/>
       <c r="D18" s="89" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E18" s="94"/>
     </row>
@@ -27221,8 +27231,8 @@
       <c r="A19" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="B19" s="95" t="s">
-        <v>452</v>
+      <c r="B19" s="93" t="s">
+        <v>702</v>
       </c>
       <c r="C19" s="92" t="s">
         <v>6</v>
@@ -27239,7 +27249,9 @@
         <f>A15+1</f>
         <v>46261</v>
       </c>
-      <c r="B20" s="95"/>
+      <c r="B20" s="109" t="s">
+        <v>708</v>
+      </c>
       <c r="C20" s="92"/>
       <c r="D20" s="93" t="s">
         <v>105</v>
@@ -27333,7 +27345,7 @@
     <row r="28" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="50"/>
       <c r="B28" s="97" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="C28" s="88"/>
       <c r="D28" s="89" t="s">
@@ -27368,7 +27380,7 @@
       </c>
       <c r="C30" s="92"/>
       <c r="D30" s="108" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="E30" s="94"/>
     </row>
@@ -27416,7 +27428,7 @@
         <v>6</v>
       </c>
       <c r="D34" s="93" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="E34" s="94" t="s">
         <v>6</v>
@@ -27830,7 +27842,7 @@
     <row r="3" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="46"/>
       <c r="B3" s="97" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="C3" s="88"/>
       <c r="D3" s="89" t="s">
@@ -27907,13 +27919,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="95" t="s">
+        <v>712</v>
+      </c>
+      <c r="C9" s="92" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="93" t="s">
         <v>713</v>
-      </c>
-      <c r="C9" s="92" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="93" t="s">
-        <v>714</v>
       </c>
       <c r="E9" s="94" t="s">
         <v>6</v>
@@ -27969,7 +27981,7 @@
         <v>10</v>
       </c>
       <c r="B14" s="95" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="C14" s="92" t="s">
         <v>6</v>
@@ -28022,7 +28034,7 @@
       </c>
       <c r="C18" s="88"/>
       <c r="D18" s="89" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="E18" s="94"/>
     </row>
@@ -28031,13 +28043,13 @@
         <v>11</v>
       </c>
       <c r="B19" s="95" t="s">
+        <v>716</v>
+      </c>
+      <c r="C19" s="92" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19" s="93" t="s">
         <v>717</v>
-      </c>
-      <c r="C19" s="92" t="s">
-        <v>6</v>
-      </c>
-      <c r="D19" s="93" t="s">
-        <v>718</v>
       </c>
       <c r="E19" s="94" t="s">
         <v>6</v>
@@ -28080,7 +28092,7 @@
     <row r="23" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="50"/>
       <c r="B23" s="97" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="C23" s="88"/>
       <c r="D23" s="89" t="s">
@@ -28093,7 +28105,7 @@
         <v>27</v>
       </c>
       <c r="B24" s="95" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="C24" s="92" t="s">
         <v>6</v>
@@ -28163,7 +28175,7 @@
         <v>6</v>
       </c>
       <c r="D29" s="93" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="E29" s="94" t="s">
         <v>6</v>
@@ -28175,7 +28187,7 @@
         <v>46270</v>
       </c>
       <c r="B30" s="95" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="C30" s="92"/>
       <c r="D30" s="93"/>
@@ -28210,7 +28222,7 @@
       </c>
       <c r="C33" s="88"/>
       <c r="D33" s="89" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="E33" s="90"/>
     </row>
@@ -28219,13 +28231,13 @@
         <v>35</v>
       </c>
       <c r="B34" s="95" t="s">
+        <v>723</v>
+      </c>
+      <c r="C34" s="92" t="s">
+        <v>6</v>
+      </c>
+      <c r="D34" s="93" t="s">
         <v>724</v>
-      </c>
-      <c r="C34" s="92" t="s">
-        <v>6</v>
-      </c>
-      <c r="D34" s="93" t="s">
-        <v>725</v>
       </c>
       <c r="E34" s="94" t="s">
         <v>6</v>
@@ -28705,7 +28717,7 @@
       </c>
       <c r="C8" s="88"/>
       <c r="D8" s="89" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="E8" s="90"/>
     </row>
@@ -28720,7 +28732,7 @@
         <v>6</v>
       </c>
       <c r="D9" s="93" t="s">
-        <v>324</v>
+        <v>261</v>
       </c>
       <c r="E9" s="94" t="s">
         <v>6</v>
@@ -28912,7 +28924,7 @@
         <v>6</v>
       </c>
       <c r="D24" s="93" t="s">
-        <v>672</v>
+        <v>726</v>
       </c>
       <c r="E24" s="94" t="s">
         <v>6</v>
@@ -28927,7 +28939,9 @@
         <v>28</v>
       </c>
       <c r="C25" s="92"/>
-      <c r="D25" s="93"/>
+      <c r="D25" s="93" t="s">
+        <v>727</v>
+      </c>
       <c r="E25" s="94"/>
     </row>
     <row r="26" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -28974,7 +28988,7 @@
         <v>6</v>
       </c>
       <c r="D29" s="93" t="s">
-        <v>108</v>
+        <v>694</v>
       </c>
       <c r="E29" s="94" t="s">
         <v>6</v>
@@ -29086,8 +29100,8 @@
       <c r="E38" s="45"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="85" orientation="landscape" r:id="rId1"/>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -29452,7 +29466,7 @@
     <row r="3" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="46"/>
       <c r="B3" s="97" t="s">
-        <v>662</v>
+        <v>602</v>
       </c>
       <c r="C3" s="88"/>
       <c r="D3" s="89" t="s">
@@ -29465,13 +29479,13 @@
         <v>5</v>
       </c>
       <c r="B4" s="95" t="s">
-        <v>63</v>
+        <v>604</v>
       </c>
       <c r="C4" s="92" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="93" t="s">
-        <v>582</v>
+        <v>637</v>
       </c>
       <c r="E4" s="94" t="s">
         <v>6</v>
@@ -29483,7 +29497,7 @@
         <v>46279</v>
       </c>
       <c r="B5" s="91" t="s">
-        <v>45</v>
+        <v>606</v>
       </c>
       <c r="C5" s="92"/>
       <c r="D5" s="93"/>
@@ -29514,11 +29528,11 @@
     <row r="8" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="50"/>
       <c r="B8" s="88" t="s">
-        <v>663</v>
+        <v>607</v>
       </c>
       <c r="C8" s="88"/>
       <c r="D8" s="89" t="s">
-        <v>53</v>
+        <v>608</v>
       </c>
       <c r="E8" s="90"/>
     </row>
@@ -29527,13 +29541,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="95" t="s">
-        <v>664</v>
+        <v>609</v>
       </c>
       <c r="C9" s="92" t="s">
         <v>6</v>
       </c>
       <c r="D9" s="93" t="s">
-        <v>324</v>
+        <v>610</v>
       </c>
       <c r="E9" s="94" t="s">
         <v>6</v>
@@ -29545,11 +29559,11 @@
         <v>46280</v>
       </c>
       <c r="B10" s="95" t="s">
-        <v>665</v>
+        <v>242</v>
       </c>
       <c r="C10" s="92"/>
       <c r="D10" s="93" t="s">
-        <v>666</v>
+        <v>36</v>
       </c>
       <c r="E10" s="94"/>
     </row>
@@ -29567,7 +29581,7 @@
     <row r="12" spans="1:5" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="47"/>
       <c r="B12" s="95" t="s">
-        <v>667</v>
+        <v>39</v>
       </c>
       <c r="C12" s="92"/>
       <c r="D12" s="93" t="s">
@@ -29578,11 +29592,11 @@
     <row r="13" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="50"/>
       <c r="B13" s="97" t="s">
-        <v>691</v>
+        <v>539</v>
       </c>
       <c r="C13" s="88"/>
       <c r="D13" s="89" t="s">
-        <v>23</v>
+        <v>352</v>
       </c>
       <c r="E13" s="90"/>
     </row>
@@ -29591,13 +29605,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="95" t="s">
-        <v>668</v>
+        <v>428</v>
       </c>
       <c r="C14" s="92" t="s">
         <v>6</v>
       </c>
       <c r="D14" s="93" t="s">
-        <v>669</v>
+        <v>611</v>
       </c>
       <c r="E14" s="94" t="s">
         <v>6</v>
@@ -29609,12 +29623,10 @@
         <v>46281</v>
       </c>
       <c r="B15" s="95" t="s">
-        <v>17</v>
+        <v>612</v>
       </c>
       <c r="C15" s="92"/>
-      <c r="D15" s="93" t="s">
-        <v>569</v>
-      </c>
+      <c r="D15" s="93"/>
       <c r="E15" s="94"/>
     </row>
     <row r="16" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -29642,11 +29654,11 @@
     <row r="18" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="50"/>
       <c r="B18" s="97" t="s">
-        <v>107</v>
+        <v>613</v>
       </c>
       <c r="C18" s="88"/>
       <c r="D18" s="89" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E18" s="94"/>
     </row>
@@ -29655,13 +29667,13 @@
         <v>11</v>
       </c>
       <c r="B19" s="95" t="s">
-        <v>121</v>
+        <v>159</v>
       </c>
       <c r="C19" s="92" t="s">
         <v>6</v>
       </c>
       <c r="D19" s="93" t="s">
-        <v>692</v>
+        <v>436</v>
       </c>
       <c r="E19" s="94" t="s">
         <v>6</v>
@@ -29673,12 +29685,10 @@
         <v>46282</v>
       </c>
       <c r="B20" s="95" t="s">
-        <v>88</v>
+        <v>614</v>
       </c>
       <c r="C20" s="92"/>
-      <c r="D20" s="93" t="s">
-        <v>670</v>
-      </c>
+      <c r="D20" s="93"/>
       <c r="E20" s="94"/>
     </row>
     <row r="21" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -29706,11 +29716,11 @@
     <row r="23" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="50"/>
       <c r="B23" s="97" t="s">
-        <v>155</v>
+        <v>257</v>
       </c>
       <c r="C23" s="88"/>
       <c r="D23" s="89" t="s">
-        <v>58</v>
+        <v>603</v>
       </c>
       <c r="E23" s="90"/>
     </row>
@@ -29719,13 +29729,13 @@
         <v>27</v>
       </c>
       <c r="B24" s="95" t="s">
-        <v>671</v>
+        <v>435</v>
       </c>
       <c r="C24" s="92" t="s">
         <v>6</v>
       </c>
       <c r="D24" s="93" t="s">
-        <v>672</v>
+        <v>605</v>
       </c>
       <c r="E24" s="94" t="s">
         <v>6</v>
@@ -29737,7 +29747,7 @@
         <v>46283</v>
       </c>
       <c r="B25" s="95" t="s">
-        <v>28</v>
+        <v>615</v>
       </c>
       <c r="C25" s="92"/>
       <c r="D25" s="93"/>
@@ -29768,11 +29778,11 @@
     <row r="28" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="50"/>
       <c r="B28" s="97" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C28" s="88"/>
       <c r="D28" s="89" t="s">
-        <v>647</v>
+        <v>107</v>
       </c>
       <c r="E28" s="94"/>
     </row>
@@ -29781,13 +29791,13 @@
         <v>30</v>
       </c>
       <c r="B29" s="95" t="s">
-        <v>648</v>
+        <v>616</v>
       </c>
       <c r="C29" s="92" t="s">
         <v>6</v>
       </c>
       <c r="D29" s="93" t="s">
-        <v>108</v>
+        <v>617</v>
       </c>
       <c r="E29" s="94" t="s">
         <v>6</v>
@@ -29799,11 +29809,11 @@
         <v>46284</v>
       </c>
       <c r="B30" s="95" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="C30" s="92"/>
       <c r="D30" s="93" t="s">
-        <v>85</v>
+        <v>462</v>
       </c>
       <c r="E30" s="94"/>
     </row>
@@ -29825,18 +29835,18 @@
       </c>
       <c r="C32" s="92"/>
       <c r="D32" s="96" t="s">
-        <v>339</v>
+        <v>618</v>
       </c>
       <c r="E32" s="94"/>
     </row>
     <row r="33" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="50"/>
       <c r="B33" s="97" t="s">
-        <v>673</v>
+        <v>636</v>
       </c>
       <c r="C33" s="88"/>
       <c r="D33" s="89" t="s">
-        <v>70</v>
+        <v>619</v>
       </c>
       <c r="E33" s="90"/>
     </row>
@@ -29845,13 +29855,13 @@
         <v>35</v>
       </c>
       <c r="B34" s="95" t="s">
-        <v>674</v>
+        <v>91</v>
       </c>
       <c r="C34" s="92" t="s">
         <v>6</v>
       </c>
       <c r="D34" s="93" t="s">
-        <v>675</v>
+        <v>620</v>
       </c>
       <c r="E34" s="94" t="s">
         <v>6</v>
@@ -29863,7 +29873,7 @@
         <v>46285</v>
       </c>
       <c r="B35" s="95" t="s">
-        <v>64</v>
+        <v>621</v>
       </c>
       <c r="C35" s="92"/>
       <c r="D35" s="93"/>

</xml_diff>